<commit_message>
Fix COPRAS chart as Excel combo: columns Q/S+/S- plus line N_i
Add s_plus and s_minus to data. Primary axis max 0.7, secondary max 120.
Combine clustered column chart with line-on-secondary per thesis spec.

Co-authored-by: sazmanfava854-sudo <sazmanfava854-sudo@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/chapter4-figures/chapter4-data.xlsx
+++ b/docs/chapter4-figures/chapter4-data.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="58">
   <si>
     <t>نمودار ۴-۱ — تغییرات شاخص Inertia و Silhouette برحسب تعداد خوشه‌ها</t>
   </si>
@@ -160,7 +160,16 @@
     <t>نمودار ۴-۱۰ — مقایسه فناوری‌ها بر اساس روش COPRAS</t>
   </si>
   <si>
-    <t>N_i</t>
+    <t>اهمیت نسبی (Q_i)</t>
+  </si>
+  <si>
+    <t>درجه مطلوبیت (N_i)</t>
+  </si>
+  <si>
+    <t>مجموع سود (S_i+)</t>
+  </si>
+  <si>
+    <t>مجموع هزینه (S_i-)</t>
   </si>
   <si>
     <t>نمودار ۴-۱۱ — مقایسه رتبه فناوری‌ها در روش‌های TOPSIS، VIKOR و COPRAS</t>
@@ -646,14 +655,11 @@
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>Q_i</c:v>
+                  <c:v>اهمیت نسبی (Q_i)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
-          <c:dLbls>
-            <c:showVal val="1"/>
-          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>'نمودار۴-۱۰'!$A$4:$A$6</c:f>
@@ -695,18 +701,136 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
+              <c:f>'نمودار۴-۱۰'!$D$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>مجموع سود (S_i+)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'نمودار۴-۱۰'!$A$4:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>LoRaWAN</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sigfox</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>NB-IoT</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'نمودار۴-۱۰'!$D$4:$D$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0.08069999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.0892</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.1087</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="2"/>
+          <c:order val="2"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'نمودار۴-۱۰'!$E$3</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>مجموع هزینه (S_i-)</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:cat>
+            <c:strRef>
+              <c:f>'نمودار۴-۱۰'!$A$4:$A$6</c:f>
+              <c:strCache>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>LoRaWAN</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sigfox</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>NB-IoT</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'نمودار۴-۱۰'!$E$4:$E$6</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>0.09379999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.1254</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.5023</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="50110001"/>
+        <c:axId val="50110002"/>
+      </c:barChart>
+      <c:lineChart>
+        <c:grouping val="straight_with_markers"/>
+        <c:ser>
+          <c:idx val="3"/>
+          <c:order val="3"/>
+          <c:tx>
+            <c:strRef>
               <c:f>'نمودار۴-۱۰'!$C$3</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
-                  <c:v>N_i</c:v>
+                  <c:v>درجه مطلوبیت (N_i)</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
           </c:tx>
-          <c:dLbls>
-            <c:showVal val="1"/>
-          </c:dLbls>
+          <c:spPr>
+            <a:ln w="31750">
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="C00000"/>
+              </a:solidFill>
+            </c:spPr>
+          </c:marker>
           <c:cat>
             <c:strRef>
               <c:f>'نمودار۴-۱۰'!$A$4:$A$6</c:f>
@@ -743,15 +867,34 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="50110001"/>
-        <c:axId val="50110002"/>
-      </c:barChart>
+        <c:marker val="1"/>
+        <c:axId val="60110001"/>
+        <c:axId val="60110002"/>
+      </c:lineChart>
       <c:catAx>
         <c:axId val="50110001"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:axPos val="b"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>فناوری</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50110002"/>
         <c:crosses val="autoZero"/>
@@ -763,18 +906,84 @@
         <c:axId val="50110002"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="0.7"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:axPos val="l"/>
         <c:majorGridlines/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>Q_i / S_i</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
         <c:numFmt formatCode="General" sourceLinked="1"/>
         <c:tickLblPos val="nextTo"/>
         <c:crossAx val="50110001"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
+      <c:valAx>
+        <c:axId val="60110002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:max val="120"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="r"/>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr rot="-5400000" vert="horz"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US"/>
+                  <a:t>N_i (%)</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:crossAx val="60110001"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:catAx>
+        <c:axId val="60110001"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="1"/>
+        <c:axPos val="b"/>
+        <c:tickLblPos val="none"/>
+        <c:crossAx val="60110002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
     </c:plotArea>
     <c:legend>
-      <c:legendPos val="r"/>
+      <c:legendPos val="b"/>
       <c:layout/>
     </c:legend>
     <c:plotVisOnly val="1"/>
@@ -2572,15 +2781,15 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>571500</xdr:colOff>
-      <xdr:row>22</xdr:row>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>533400</xdr:colOff>
+      <xdr:row>24</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -3388,33 +3597,40 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
-    <col min="2" max="3" width="14.7109375" customWidth="1"/>
+    <col min="2" max="5" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="36" customHeight="1">
+    <row r="1" spans="1:5" ht="36" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="E1" s="1"/>
+    </row>
+    <row r="3" spans="1:5">
       <c r="A3" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4">
+        <v>45</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -3424,8 +3640,14 @@
       <c r="C4">
         <v>100</v>
       </c>
-    </row>
-    <row r="5" spans="1:4">
+      <c r="D4">
+        <v>0.08069999999999999</v>
+      </c>
+      <c r="E4">
+        <v>0.09379999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -3435,8 +3657,14 @@
       <c r="C5">
         <v>81.2</v>
       </c>
-    </row>
-    <row r="6" spans="1:4">
+      <c r="D5">
+        <v>0.0892</v>
+      </c>
+      <c r="E5">
+        <v>0.1254</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
       <c r="A6" t="s">
         <v>37</v>
       </c>
@@ -3446,10 +3674,16 @@
       <c r="C6">
         <v>39.3</v>
       </c>
+      <c r="D6">
+        <v>0.1087</v>
+      </c>
+      <c r="E6">
+        <v>0.5023</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -3467,7 +3701,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3478,13 +3712,13 @@
         <v>33</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -3549,7 +3783,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="36" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -3557,15 +3791,15 @@
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="2" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B4">
         <v>1</v>
@@ -3573,7 +3807,7 @@
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B5">
         <v>1</v>
@@ -3581,7 +3815,7 @@
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B6">
         <v>1</v>

</xml_diff>